<commit_message>
Update berita 2026-08-04 10:33 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-30.xlsx
+++ b/data/berita_antara_2026-07-30.xlsx
@@ -511,33 +511,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
+          <t>IHSG menguat dipicu "risk on" pasar seiring The Fed tahan suku bunga</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
+          <t>Thu, 30 Jul 2026 09:48:24 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis bergerak menguat dipicu oleh sikap risk ...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
+          <t>https://www.antaranews.com/berita/5672087/ihsg-menguat-dipicu-risk-on-pasar-seiring-the-fed-tahan-suku-bunga</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -549,33 +549,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
+          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
+          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
+          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
+          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -587,33 +587,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
+          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
+          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
+          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
+          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -630,28 +630,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
+          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
+          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
+          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
+          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -668,28 +668,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
+          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
+          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
+          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -706,28 +706,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
+          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
+          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
+          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -744,28 +744,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>United Tractors cetak pendapatan Rp58,3 triliun di semester I-2026</t>
+          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 12:29:10 +0700</t>
+          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Perusahaan grup PT Astra International Tbk (ASII) yaitu PT United Tractors Tbk (UNTR) membukukan pendapatan bersih ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672283/united-tractors-cetak-pendapatan-rp583-triliun-di-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/16/1000566369_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -782,28 +782,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IHSG menguat dipicu "risk on" pasar seiring The Fed tahan suku bunga</t>
+          <t>United Tractors cetak pendapatan Rp58,3 triliun di semester I-2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 09:48:24 +0700</t>
+          <t>Thu, 30 Jul 2026 12:29:10 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis bergerak menguat dipicu oleh sikap risk ...</t>
+          <t>Perusahaan grup PT Astra International Tbk (ASII) yaitu PT United Tractors Tbk (UNTR) membukukan pendapatan bersih ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672087/ihsg-menguat-dipicu-risk-on-pasar-seiring-the-fed-tahan-suku-bunga</t>
+          <t>https://www.antaranews.com/berita/5672283/united-tractors-cetak-pendapatan-rp583-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/16/1000566369_1.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>

<commit_message>
Update berita 2026-08-04 10:56 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-30.xlsx
+++ b/data/berita_antara_2026-07-30.xlsx
@@ -549,33 +549,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
+          <t>United Tractors cetak pendapatan Rp58,3 triliun di semester I-2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
+          <t>Thu, 30 Jul 2026 12:29:10 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
+          <t>Perusahaan grup PT Astra International Tbk (ASII) yaitu PT United Tractors Tbk (UNTR) membukukan pendapatan bersih ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
+          <t>https://www.antaranews.com/berita/5672283/united-tractors-cetak-pendapatan-rp583-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/16/1000566369_1.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -587,33 +587,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
+          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
+          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
+          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
+          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -625,33 +625,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
+          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
+          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
+          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
+          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -668,28 +668,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
+          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
+          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
+          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
+          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -706,28 +706,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
+          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
+          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
+          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -744,28 +744,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
+          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
+          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
+          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -782,28 +782,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>United Tractors cetak pendapatan Rp58,3 triliun di semester I-2026</t>
+          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 12:29:10 +0700</t>
+          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Perusahaan grup PT Astra International Tbk (ASII) yaitu PT United Tractors Tbk (UNTR) membukukan pendapatan bersih ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672283/united-tractors-cetak-pendapatan-rp583-triliun-di-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/16/1000566369_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>

<commit_message>
Update berita 2026-08-04 12:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-30.xlsx
+++ b/data/berita_antara_2026-07-30.xlsx
@@ -587,33 +587,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
+          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
+          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
+          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
+          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -625,33 +625,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
+          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
+          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
+          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -668,28 +668,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PU uji coba irigasi Pante Lhong Aceh untuk aliri 6.562 hektare sawah</t>
+          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:28:11 +0700</t>
+          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Menteri Pekerjaan Umum (PU) Dody Hanggodo melakukan uji coba irigasi Pante Lhong Kabupaten Bireuen, Aceh yang telah ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672783/pu-uji-coba-irigasi-pante-lhong-aceh-untuk-aliri-6562-hektare-sawah</t>
+          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IMG-20260730-WA0014_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -706,28 +706,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IHSG ditutup menguat ditopang musim laporan keuangan emiten</t>
+          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 17:05:56 +0700</t>
+          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Kamis sore ditutup menguat ditopang oleh musim ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672741/ihsg-ditutup-menguat-ditopang-musim-laporan-keuangan-emiten</t>
+          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/25/pembukaan-ihsg-usai-libur-lebaran-2760782.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -739,33 +739,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OJK tuntaskan pemeriksaan 17 kasus manipulasi di pasar modal</t>
+          <t>20 ide tema 17 Agustus 2026 yang kreatif, unik, dan penuh makna untuk HUT ke-81 RI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 16:26:08 +0700</t>
+          <t>Thu, 30 Jul 2026 23:34:21 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan telah menyelesaikan pemeriksaan atas sebanyak 17 kasus terkait pelanggaran ...</t>
+          <t>Perayaan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 tinggal menghitung hari. ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672663/ojk-tuntaskan-pemeriksaan-17-kasus-manipulasi-di-pasar-modal</t>
+          <t>https://www.antaranews.com/berita/5673507/20-ide-tema-17-agustus-2026-yang-kreatif-unik-dan-penuh-makna-untuk-hut-ke-81-ri</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/IMG-20260630-WA0035.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -777,33 +777,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OJK ungkap 7 manajer investasi andil peluncuran ETF Emas di 10 Agustus</t>
+          <t>6 titik shuttle bus gratis GIIAS 2026 ke ICE BSD, cek lokasi &amp; jadwalnya</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 14:07:07 +0700</t>
+          <t>Thu, 30 Jul 2026 18:17:21 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan sebanyak lima sampai tujuh Manajer Investasi (MI) akan turut berpartisipasi ...</t>
+          <t>Penyelenggara GAIKINDO Indonesia International Auto Show (GIIAS) 2026 kembali menyediakan layanan shuttle bus gratis ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5672456/ojk-ungkap-7-manajer-investasi-andil-peluncuran-etf-emas-di-10-agustus</t>
+          <t>https://otomotif.antaranews.com/berita/5672876/6-titik-shuttle-bus-gratis-giias-2026-ke-ice-bsd-cek-lokasi-jadwalnya</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/06/IMG-20260406-WA0035_copy_1280x732.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1404.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>